<commit_message>
Changes in the statistical analysis
</commit_message>
<xml_diff>
--- a/2d/results/best_unet_filter_distance_max/best_unet.xlsx
+++ b/2d/results/best_unet_filter_distance_max/best_unet.xlsx
@@ -535,10 +535,10 @@
         <v>140</v>
       </c>
       <c r="C2" t="n">
+        <v>23.71181140275874</v>
+      </c>
+      <c r="D2" t="n">
         <v>14.86606874731851</v>
-      </c>
-      <c r="D2" t="n">
-        <v>23.71181140275874</v>
       </c>
       <c r="E2" t="n">
         <v>36.05318827440322</v>
@@ -596,10 +596,10 @@
         <v>141</v>
       </c>
       <c r="C3" t="n">
+        <v>14.30034964607509</v>
+      </c>
+      <c r="D3" t="n">
         <v>17.26991603917055</v>
-      </c>
-      <c r="D3" t="n">
-        <v>14.30034964607509</v>
       </c>
       <c r="E3" t="n">
         <v>29.3671181690799</v>
@@ -657,10 +657,10 @@
         <v>149</v>
       </c>
       <c r="C4" t="n">
+        <v>12.36931687685298</v>
+      </c>
+      <c r="D4" t="n">
         <v>8.944271909999159</v>
-      </c>
-      <c r="D4" t="n">
-        <v>12.36931687685298</v>
       </c>
       <c r="E4" t="n">
         <v>18.10344827586206</v>
@@ -718,10 +718,10 @@
         <v>160</v>
       </c>
       <c r="C5" t="n">
+        <v>20.24845673131659</v>
+      </c>
+      <c r="D5" t="n">
         <v>16.56804152578089</v>
-      </c>
-      <c r="D5" t="n">
-        <v>20.24845673131659</v>
       </c>
       <c r="E5" t="n">
         <v>39.67122657776761</v>
@@ -779,10 +779,10 @@
         <v>170</v>
       </c>
       <c r="C6" t="n">
+        <v>14.8660687473185</v>
+      </c>
+      <c r="D6" t="n">
         <v>5.315072906367329</v>
-      </c>
-      <c r="D6" t="n">
-        <v>14.8660687473185</v>
       </c>
       <c r="E6" t="n">
         <v>18.52228435858337</v>
@@ -840,10 +840,10 @@
         <v>184</v>
       </c>
       <c r="C7" t="n">
+        <v>14.56021977856104</v>
+      </c>
+      <c r="D7" t="n">
         <v>12.02081528017131</v>
-      </c>
-      <c r="D7" t="n">
-        <v>14.56021977856104</v>
       </c>
       <c r="E7" t="n">
         <v>30.32128514056221</v>
@@ -901,10 +901,10 @@
         <v>190</v>
       </c>
       <c r="C8" t="n">
+        <v>11.71537451385999</v>
+      </c>
+      <c r="D8" t="n">
         <v>7.648529270389178</v>
-      </c>
-      <c r="D8" t="n">
-        <v>11.71537451385999</v>
       </c>
       <c r="E8" t="n">
         <v>32.2371886522688</v>
@@ -962,10 +962,10 @@
         <v>198</v>
       </c>
       <c r="C9" t="n">
+        <v>25.46566315649369</v>
+      </c>
+      <c r="D9" t="n">
         <v>15.20690632574555</v>
-      </c>
-      <c r="D9" t="n">
-        <v>25.46566315649369</v>
       </c>
       <c r="E9" t="n">
         <v>22.80382775119626</v>
@@ -1023,10 +1023,10 @@
         <v>199</v>
       </c>
       <c r="C10" t="n">
+        <v>15.43534904043313</v>
+      </c>
+      <c r="D10" t="n">
         <v>12.17579566188592</v>
-      </c>
-      <c r="D10" t="n">
-        <v>15.43534904043313</v>
       </c>
       <c r="E10" t="n">
         <v>37.75196774812821</v>
@@ -1084,10 +1084,10 @@
         <v>100</v>
       </c>
       <c r="C11" t="n">
+        <v>20.71834935510066</v>
+      </c>
+      <c r="D11" t="n">
         <v>8.200609733428356</v>
-      </c>
-      <c r="D11" t="n">
-        <v>20.71834935510066</v>
       </c>
       <c r="E11" t="n">
         <v>21.25000000000003</v>
@@ -1145,10 +1145,10 @@
         <v>106</v>
       </c>
       <c r="C12" t="n">
+        <v>17.08800749063506</v>
+      </c>
+      <c r="D12" t="n">
         <v>7.211102550927979</v>
-      </c>
-      <c r="D12" t="n">
-        <v>17.08800749063506</v>
       </c>
       <c r="E12" t="n">
         <v>22.38104562365379</v>
@@ -1206,10 +1206,10 @@
         <v>111</v>
       </c>
       <c r="C13" t="n">
+        <v>11.88486432400471</v>
+      </c>
+      <c r="D13" t="n">
         <v>7.433034373659253</v>
-      </c>
-      <c r="D13" t="n">
-        <v>11.88486432400471</v>
       </c>
       <c r="E13" t="n">
         <v>20.18779342723001</v>
@@ -1267,10 +1267,10 @@
         <v>135</v>
       </c>
       <c r="C14" t="n">
+        <v>20.13082213919739</v>
+      </c>
+      <c r="D14" t="n">
         <v>11.88486432400471</v>
-      </c>
-      <c r="D14" t="n">
-        <v>20.13082213919739</v>
       </c>
       <c r="E14" t="n">
         <v>34.79035737735677</v>
@@ -1328,10 +1328,10 @@
         <v>990</v>
       </c>
       <c r="C15" t="n">
+        <v>18.78829422805594</v>
+      </c>
+      <c r="D15" t="n">
         <v>10.12422836565829</v>
-      </c>
-      <c r="D15" t="n">
-        <v>18.78829422805594</v>
       </c>
       <c r="E15" t="n">
         <v>28.46028239362212</v>
@@ -1389,10 +1389,10 @@
         <v>920</v>
       </c>
       <c r="C16" t="n">
+        <v>26.73013280924732</v>
+      </c>
+      <c r="D16" t="n">
         <v>13.00000000000001</v>
-      </c>
-      <c r="D16" t="n">
-        <v>26.73013280924732</v>
       </c>
       <c r="E16" t="n">
         <v>33.66436384571112</v>

</xml_diff>